<commit_message>
Added values for preconditions, method inputs, and expected results for each test in the test plan.
</commit_message>
<xml_diff>
--- a/tests/A01_pixell_test_plan_client.xlsx
+++ b/tests/A01_pixell_test_plan_client.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27728"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dkwarkentin\Documents\Course Folders\2-Intermediate Software Development\Code\Assignments 2024 Spring\Assignment 1\tests\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\Documents\rrc_polytech\winter_2025\isd_2025\Assignments\isd_project\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ECD6C5C-0BF7-4659-811B-1D416A6C1BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8AAAD5-0B69-46D2-A9F1-2C01F58933A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="43155" yWindow="0" windowWidth="14550" windowHeight="15585" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
   <si>
     <t>Software Development Team - Unit Test Plan</t>
   </si>
@@ -264,13 +264,87 @@
   </si>
   <si>
     <t>Add more rows as necessary</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>client_number = 1234
+first_name = "Xavier"
+last_name = "Balzer"
+email_address = "xbalzer@rrc.ca"</t>
+  </si>
+  <si>
+    <t>Object is initialized with the correct state.</t>
+  </si>
+  <si>
+    <t>ValueError: Client number must be numeric.</t>
+  </si>
+  <si>
+    <t>ValueError: First name cannot be blank.</t>
+  </si>
+  <si>
+    <t>ValueError: Last name cannot be blank.</t>
+  </si>
+  <si>
+    <t>Object initialized.
+client_number = 1234
+first_name = "Xavier"
+last_name = "Balzer"
+email_address = "xbalzer@rrc.ca"</t>
+  </si>
+  <si>
+    <t>client_number = 1234
+first_name = "Xavier"
+last_name = "Balzer"
+email_address = "invalid"</t>
+  </si>
+  <si>
+    <t>email_address =
+ "email@pixell-river.com"</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> "1234"</t>
+  </si>
+  <si>
+    <t>"Xavier"</t>
+  </si>
+  <si>
+    <t>"Balzer"</t>
+  </si>
+  <si>
+    <t>"Balzer, Xavier [1234] - xbalzer@rrc.ca"</t>
+  </si>
+  <si>
+    <t>client_number = 1234
+first_name = "Xavier"
+last_name = "   "
+email_address = "xbalzer@rrc.ca"</t>
+  </si>
+  <si>
+    <t>client_number = 1234
+first_name = "    "
+last_name = "Balzer"
+email_address = "xbalzer@rrc.ca"</t>
+  </si>
+  <si>
+    <t>client_number = "string"
+first_name = "Xavier"
+last_name = "Balzer"
+email_address = "xbalzer@rrc.ca"</t>
+  </si>
+  <si>
+    <t>Xavier Balzer</t>
+  </si>
+  <si>
+    <t>xbalzer@rrc.ca</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -331,6 +405,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -504,10 +586,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -558,8 +641,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
@@ -1086,7 +1173,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DADEBCC4-BB44-48CD-B9AB-1E2FD3EE0EEB}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="12.7109375" customWidth="1"/>
     <col min="3" max="3" width="22.28515625" customWidth="1"/>
@@ -1096,7 +1183,7 @@
     <col min="7" max="7" width="26.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" thickBot="1"/>
+    <row r="1" spans="1:7" ht="15.75" thickBot="1"/>
     <row r="2" spans="1:7" ht="73.150000000000006" customHeight="1" thickBot="1">
       <c r="B2" s="2" t="e" vm="1">
         <v>#VALUE!</v>
@@ -1109,14 +1196,16 @@
       <c r="F2" s="13"/>
       <c r="G2" s="14"/>
     </row>
-    <row r="3" spans="1:7" ht="15" thickBot="1">
+    <row r="3" spans="1:7" ht="15.75" thickBot="1">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15"/>
+      <c r="C3" s="15" t="s">
+        <v>43</v>
+      </c>
       <c r="D3" s="16"/>
     </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1">
+    <row r="4" spans="1:7" ht="15.75" thickBot="1">
       <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
@@ -1159,9 +1248,15 @@
       <c r="D7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
+      <c r="E7" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="8" spans="1:7" ht="66" customHeight="1">
       <c r="A8" s="4"/>
@@ -1174,9 +1269,15 @@
       <c r="D8" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
+      <c r="E8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="9" spans="1:7" ht="66" customHeight="1">
       <c r="A9" s="4"/>
@@ -1189,9 +1290,15 @@
       <c r="D9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
+      <c r="E9" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="10" spans="1:7" ht="66" customHeight="1">
       <c r="A10" s="4"/>
@@ -1204,9 +1311,15 @@
       <c r="D10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
+      <c r="E10" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="11" spans="1:7" ht="66" customHeight="1">
       <c r="A11" s="4"/>
@@ -1219,11 +1332,17 @@
       <c r="D11" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-    </row>
-    <row r="12" spans="1:7" ht="31.15" customHeight="1">
+      <c r="E11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="105">
       <c r="B12" s="11">
         <v>6</v>
       </c>
@@ -1233,11 +1352,17 @@
       <c r="D12" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-    </row>
-    <row r="13" spans="1:7" ht="31.15" customHeight="1">
+      <c r="E12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="105">
       <c r="B13" s="9">
         <v>7</v>
       </c>
@@ -1247,11 +1372,17 @@
       <c r="D13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-    </row>
-    <row r="14" spans="1:7" ht="31.15" customHeight="1">
+      <c r="E13" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="105">
       <c r="B14" s="11">
         <v>8</v>
       </c>
@@ -1261,11 +1392,17 @@
       <c r="D14" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-    </row>
-    <row r="15" spans="1:7" ht="31.15" customHeight="1">
+      <c r="E14" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="105">
       <c r="B15" s="11">
         <v>9</v>
       </c>
@@ -1275,11 +1412,17 @@
       <c r="D15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-    </row>
-    <row r="16" spans="1:7" ht="31.15" customHeight="1">
+      <c r="E15" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="105">
       <c r="B16" s="9">
         <v>10</v>
       </c>
@@ -1289,9 +1432,15 @@
       <c r="D16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
+      <c r="E16" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="17" spans="2:7" ht="31.15" customHeight="1">
       <c r="B17" s="11">
@@ -1430,10 +1579,14 @@
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="B30:G30"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="G15" r:id="rId1" xr:uid="{EDA83E8F-4CDA-4EE6-83B4-62DB03B1F318}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed expected outcomes for the email accessor and string representation
</commit_message>
<xml_diff>
--- a/tests/A01_pixell_test_plan_client.xlsx
+++ b/tests/A01_pixell_test_plan_client.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\Documents\rrc_polytech\winter_2025\isd_2025\Assignments\isd_project\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8AAAD5-0B69-46D2-A9F1-2C01F58933A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F6C568-454A-4EA3-88D5-174B134C5C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43155" yWindow="0" windowWidth="14550" windowHeight="15585" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14670" windowHeight="15585" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -313,9 +313,6 @@
     <t>"Balzer"</t>
   </si>
   <si>
-    <t>"Balzer, Xavier [1234] - xbalzer@rrc.ca"</t>
-  </si>
-  <si>
     <t>client_number = 1234
 first_name = "Xavier"
 last_name = "   "
@@ -338,6 +335,9 @@
   </si>
   <si>
     <t>xbalzer@rrc.ca</t>
+  </si>
+  <si>
+    <t>f"Balzer, Xavier [1234] - xbalzer@rrc.ca\n"</t>
   </si>
 </sst>
 </file>
@@ -617,6 +617,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -640,9 +643,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1188,31 +1188,31 @@
       <c r="B2" s="2" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="15"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickBot="1">
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="D3" s="16"/>
+      <c r="C3" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:7" ht="15.75" thickBot="1">
       <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="18"/>
+      <c r="D4" s="19"/>
     </row>
     <row r="5" spans="1:7">
       <c r="B5" s="1"/>
@@ -1273,7 +1273,7 @@
         <v>27</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>30</v>
@@ -1294,7 +1294,7 @@
         <v>27</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>31</v>
@@ -1315,7 +1315,7 @@
         <v>27</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>32</v>
@@ -1418,8 +1418,8 @@
       <c r="F15" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G15" s="20" t="s">
-        <v>44</v>
+      <c r="G15" s="12" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="105">
@@ -1439,7 +1439,7 @@
         <v>27</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="2:7" ht="31.15" customHeight="1">
@@ -1563,14 +1563,14 @@
       <c r="G28" s="3"/>
     </row>
     <row r="30" spans="2:7">
-      <c r="B30" s="19" t="s">
+      <c r="B30" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>